<commit_message>
Fix PDF scraper column alignment issue
Problem: The regex was trying to skip an "index_level" that wasn't
being captured (no % sign), causing all columns to shift left by 1.
Result: 1-month data was actually showing 3-month data.

Fix:
- Removed index_level from output (not needed by merge_sp_data.py)
- Extract only percentage values (with % sign)
- Map directly: percentages[0]=1_mo, percentages[1]=3_mos, etc.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual_data.xlsx
+++ b/manual_data.xlsx
@@ -643,23 +643,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9.960000000000001</v>
+        <v>17.11</v>
       </c>
       <c r="C2" t="n">
-        <v>37.38</v>
+        <v>126.95</v>
       </c>
       <c r="D2" t="n">
-        <v>100.31</v>
+        <v>49.54</v>
       </c>
       <c r="E2" t="n">
-        <v>47.8</v>
+        <v>22.86</v>
       </c>
       <c r="F2" t="n">
-        <v>21.16</v>
-      </c>
-      <c r="G2" t="n">
-        <v>24.57</v>
-      </c>
+        <v>23.47</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -673,23 +671,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-2.66</v>
+        <v>-1.01</v>
       </c>
       <c r="C3" t="n">
-        <v>-3.05</v>
+        <v>10.32</v>
       </c>
       <c r="D3" t="n">
-        <v>5.47</v>
+        <v>11.39</v>
       </c>
       <c r="E3" t="n">
-        <v>9.710000000000001</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>9.869999999999999</v>
-      </c>
-      <c r="G3" t="n">
-        <v>9.460000000000001</v>
-      </c>
+        <v>9.31</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -703,23 +699,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-3.85</v>
+        <v>-1.4</v>
       </c>
       <c r="C4" t="n">
-        <v>-6.28</v>
+        <v>9.24</v>
       </c>
       <c r="D4" t="n">
-        <v>0.77</v>
+        <v>15.03</v>
       </c>
       <c r="E4" t="n">
-        <v>12.71</v>
+        <v>8.84</v>
       </c>
       <c r="F4" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="G4" t="n">
-        <v>8.119999999999999</v>
-      </c>
+        <v>7.91</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -733,23 +727,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-2.3</v>
+        <v>-6.45</v>
       </c>
       <c r="C5" t="n">
-        <v>-6.07</v>
+        <v>10.56</v>
       </c>
       <c r="D5" t="n">
-        <v>9.77</v>
+        <v>10.99</v>
       </c>
       <c r="E5" t="n">
-        <v>11.18</v>
+        <v>10.17</v>
       </c>
       <c r="F5" t="n">
-        <v>10.73</v>
-      </c>
-      <c r="G5" t="n">
-        <v>3.38</v>
-      </c>
+        <v>2.63</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -763,23 +755,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.64</v>
+        <v>-11.69</v>
       </c>
       <c r="C6" t="n">
-        <v>-10.12</v>
+        <v>4.09</v>
       </c>
       <c r="D6" t="n">
-        <v>6.12</v>
+        <v>16.41</v>
       </c>
       <c r="E6" t="n">
-        <v>14.64</v>
+        <v>9.32</v>
       </c>
       <c r="F6" t="n">
-        <v>10.12</v>
-      </c>
-      <c r="G6" t="n">
-        <v>11.46</v>
-      </c>
+        <v>10.45</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -793,23 +783,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.64</v>
+        <v>-1.02</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.71</v>
+        <v>2.01</v>
       </c>
       <c r="D7" t="n">
-        <v>5.59</v>
+        <v>0.73</v>
       </c>
       <c r="E7" t="n">
-        <v>1.08</v>
+        <v>1.42</v>
       </c>
       <c r="F7" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="G7" t="n">
-        <v>7.19</v>
-      </c>
+        <v>6.16</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -823,23 +811,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.57</v>
+        <v>1.15</v>
       </c>
       <c r="C8" t="n">
-        <v>-7.01</v>
+        <v>3.21</v>
       </c>
       <c r="D8" t="n">
-        <v>5.44</v>
+        <v>-2.63</v>
       </c>
       <c r="E8" t="n">
-        <v>-3.37</v>
+        <v>6.7</v>
       </c>
       <c r="F8" t="n">
-        <v>6.91</v>
-      </c>
-      <c r="G8" t="n">
-        <v>4.24</v>
-      </c>
+        <v>4.86</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -853,23 +839,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-6.53</v>
+        <v>-1.91</v>
       </c>
       <c r="C9" t="n">
-        <v>-6.46</v>
+        <v>12.05</v>
       </c>
       <c r="D9" t="n">
-        <v>3.85</v>
+        <v>18.56</v>
       </c>
       <c r="E9" t="n">
-        <v>15.86</v>
+        <v>16.2</v>
       </c>
       <c r="F9" t="n">
-        <v>15.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>8.69</v>
-      </c>
+        <v>8.66</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -883,23 +867,21 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.99</v>
+        <v>-9.880000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>-6.97</v>
+        <v>-23.66</v>
       </c>
       <c r="D10" t="n">
-        <v>-19.31</v>
+        <v>-5.22</v>
       </c>
       <c r="E10" t="n">
-        <v>-4.3</v>
+        <v>-2.87</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.4</v>
-      </c>
-      <c r="G10" t="n">
-        <v>7.93</v>
-      </c>
+        <v>7.08</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -913,23 +895,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-3.8</v>
+        <v>-4.56</v>
       </c>
       <c r="C11" t="n">
-        <v>-6.45</v>
+        <v>3.95</v>
       </c>
       <c r="D11" t="n">
-        <v>0.83</v>
+        <v>12.29</v>
       </c>
       <c r="E11" t="n">
-        <v>10.85</v>
+        <v>9.34</v>
       </c>
       <c r="F11" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="G11" t="n">
-        <v>8.31</v>
-      </c>
+        <v>7.93</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -943,23 +923,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-11.58</v>
+        <v>-26.01</v>
       </c>
       <c r="C12" t="n">
-        <v>-20.71</v>
+        <v>-20.8</v>
       </c>
       <c r="D12" t="n">
-        <v>-17.08</v>
+        <v>15.96</v>
       </c>
       <c r="E12" t="n">
-        <v>17.32</v>
+        <v>0.22</v>
       </c>
       <c r="F12" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="G12" t="n">
-        <v>13.05</v>
-      </c>
+        <v>11.64</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -973,23 +951,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.55</v>
+        <v>12.99</v>
       </c>
       <c r="C13" t="n">
-        <v>12.37</v>
+        <v>36.21</v>
       </c>
       <c r="D13" t="n">
-        <v>21.95</v>
+        <v>10.94</v>
       </c>
       <c r="E13" t="n">
-        <v>8.27</v>
+        <v>11.92</v>
       </c>
       <c r="F13" t="n">
-        <v>12.37</v>
-      </c>
-      <c r="G13" t="n">
-        <v>16.17</v>
-      </c>
+        <v>16.78</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1003,23 +979,21 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-2.06</v>
+        <v>-2.58</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.84</v>
+        <v>13.22</v>
       </c>
       <c r="D14" t="n">
-        <v>14.88</v>
+        <v>11.12</v>
       </c>
       <c r="E14" t="n">
-        <v>11.07</v>
+        <v>14.39</v>
       </c>
       <c r="F14" t="n">
-        <v>13.37</v>
-      </c>
-      <c r="G14" t="n">
-        <v>9.35</v>
-      </c>
+        <v>8.880000000000001</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1033,23 +1007,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-1.27</v>
+        <v>8.34</v>
       </c>
       <c r="C15" t="n">
-        <v>11.52</v>
+        <v>39.34</v>
       </c>
       <c r="D15" t="n">
-        <v>27.42</v>
+        <v>17.12</v>
       </c>
       <c r="E15" t="n">
-        <v>12.04</v>
+        <v>12.34</v>
       </c>
       <c r="F15" t="n">
-        <v>10.76</v>
-      </c>
-      <c r="G15" t="n">
-        <v>12.35</v>
-      </c>
+        <v>13.32</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1063,23 +1035,21 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.31</v>
+        <v>-0.04</v>
       </c>
       <c r="C16" t="n">
-        <v>1.59</v>
+        <v>18.35</v>
       </c>
       <c r="D16" t="n">
-        <v>15.32</v>
+        <v>12.75</v>
       </c>
       <c r="E16" t="n">
-        <v>11.44</v>
+        <v>10.27</v>
       </c>
       <c r="F16" t="n">
-        <v>11.27</v>
-      </c>
-      <c r="G16" t="n">
-        <v>12.31</v>
-      </c>
+        <v>11.95</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1093,23 +1063,21 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-1.48</v>
+        <v>1.8</v>
       </c>
       <c r="C17" t="n">
-        <v>3.84</v>
+        <v>24.96</v>
       </c>
       <c r="D17" t="n">
-        <v>19.43</v>
+        <v>13.44</v>
       </c>
       <c r="E17" t="n">
-        <v>11.49</v>
+        <v>6.85</v>
       </c>
       <c r="F17" t="n">
-        <v>7.13</v>
-      </c>
-      <c r="G17" t="n">
-        <v>8.9</v>
-      </c>
+        <v>8.640000000000001</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>2026-01-19</t>

</xml_diff>

<commit_message>
Add reset_commentary.bat for fresh monthly template
- Creates blank commentary.md with all section headers
- Backs up existing commentary before resetting
- Updated WORKFLOW.md with review-then-write pattern
- Added commentary_backup_*.md to .gitignore

Workflow: Generate preview → Review data → Write commentary → Regenerate

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual_data.xlsx
+++ b/manual_data.xlsx
@@ -643,21 +643,23 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="C2" t="n">
         <v>17.11</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>126.95</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>49.54</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>22.86</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>23.47</v>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -671,21 +673,23 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C3" t="n">
         <v>-1.01</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>10.32</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>11.39</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>9.890000000000001</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>9.31</v>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -699,21 +703,23 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="C4" t="n">
         <v>-1.4</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>9.24</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>15.03</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>8.84</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>7.91</v>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -727,21 +733,23 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>-3.11</v>
+      </c>
+      <c r="C5" t="n">
         <v>-6.45</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>10.56</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>10.99</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>10.17</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>2.63</v>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -755,21 +763,23 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>-2.65</v>
+      </c>
+      <c r="C6" t="n">
         <v>-11.69</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>4.09</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>16.41</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>9.32</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>10.45</v>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -783,21 +793,23 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>-2.77</v>
+      </c>
+      <c r="C7" t="n">
         <v>-1.02</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>2.01</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>0.73</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>1.42</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>6.16</v>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -811,21 +823,23 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>-1.87</v>
+      </c>
+      <c r="C8" t="n">
         <v>1.15</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>3.21</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>-2.63</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>6.7</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>4.86</v>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -839,21 +853,23 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="C9" t="n">
         <v>-1.91</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>12.05</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>18.56</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>16.2</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>8.66</v>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -867,21 +883,23 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>-7.14</v>
+      </c>
+      <c r="C10" t="n">
         <v>-9.880000000000001</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>-23.66</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>-5.22</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>-2.87</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>7.08</v>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -895,21 +913,23 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="C11" t="n">
         <v>-4.56</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>3.95</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>12.29</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>9.34</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>7.93</v>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -923,21 +943,23 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>-8.68</v>
+      </c>
+      <c r="C12" t="n">
         <v>-26.01</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>-20.8</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>15.96</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.22</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>11.64</v>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -951,21 +973,23 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="C13" t="n">
         <v>12.99</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>36.21</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>10.94</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>11.92</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>16.78</v>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -979,21 +1003,23 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="C14" t="n">
         <v>-2.58</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>13.22</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>11.12</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>14.39</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>8.880000000000001</v>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1007,21 +1033,23 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="C15" t="n">
         <v>8.34</v>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>39.34</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>17.12</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>12.34</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>13.32</v>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1035,21 +1063,23 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="C16" t="n">
         <v>-0.04</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>18.35</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>12.75</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>10.27</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>11.95</v>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>2026-01-19</t>
@@ -1063,21 +1093,23 @@
         </is>
       </c>
       <c r="B17" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="C17" t="n">
         <v>1.8</v>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>24.96</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>13.44</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>6.85</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>8.640000000000001</v>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>2026-01-19</t>

</xml_diff>

<commit_message>
Update GICS to January 2026 data, strip header in Streamlit
- Update GICS sector data from PDF scraper (Jan 2026)
- Streamlit now strips header/nav, shows article content only
- Regenerate newsletter with updated GICS values

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual_data.xlsx
+++ b/manual_data.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="CPI_Benchmarks" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,14 +12,14 @@
     <sheet name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
@@ -32,7 +31,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,24 +54,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -432,41 +445,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Fund Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1 Mth</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>3 Mth</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>1 Yr pa</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>3 Yr pa</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>5 Yr pa</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -479,21 +497,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.01</v>
+        <v>0.96</v>
       </c>
       <c r="C2" t="n">
-        <v>0.361336946702795</v>
+        <v>0.97</v>
       </c>
       <c r="D2" t="n">
         <v>3.81021594684385</v>
       </c>
       <c r="E2" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>45991</v>
-      </c>
-      <c r="G2" t="inlineStr">
+        <v>3.02997354209706</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3.16635878181464</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Update monthly from ABS</t>
         </is>
@@ -506,21 +527,24 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07333333333333333</v>
+        <v>1.043333333333333</v>
       </c>
       <c r="C3" t="n">
-        <v>0.611336946702795</v>
+        <v>1.22</v>
       </c>
       <c r="D3" t="n">
         <v>4.81021594684385</v>
       </c>
       <c r="E3" t="n">
-        <v>4.779999999999999</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>45991</v>
-      </c>
-      <c r="G3" t="inlineStr">
+        <v>4.029973542097061</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.16635878181464</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>CPI + 1%</t>
         </is>
@@ -533,21 +557,24 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1566666666666666</v>
+        <v>1.126666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.861336946702795</v>
+        <v>1.47</v>
       </c>
       <c r="D4" t="n">
         <v>5.81021594684385</v>
       </c>
       <c r="E4" t="n">
-        <v>5.779999999999999</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>45991</v>
-      </c>
-      <c r="G4" t="inlineStr">
+        <v>5.029973542097061</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5.16635878181464</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>CPI + 2%</t>
         </is>
@@ -560,21 +587,24 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.24</v>
+        <v>1.21</v>
       </c>
       <c r="C5" t="n">
-        <v>1.111336946702795</v>
+        <v>1.72</v>
       </c>
       <c r="D5" t="n">
         <v>6.81021594684385</v>
       </c>
       <c r="E5" t="n">
-        <v>6.779999999999999</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>45991</v>
-      </c>
-      <c r="G5" t="inlineStr">
+        <v>6.029973542097061</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6.16635878181464</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>CPI + 3%</t>
         </is>
@@ -595,42 +625,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Fund Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1 Mth</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>3 Mth</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>1 Yr pa</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>3 Yr pa</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>5 Yr pa</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>10 Yr pa</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
@@ -643,26 +673,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.89</v>
+        <v>10.99</v>
       </c>
       <c r="C2" t="n">
-        <v>17.11</v>
+        <v>30.46</v>
       </c>
       <c r="D2" t="n">
-        <v>126.95</v>
+        <v>118.68</v>
       </c>
       <c r="E2" t="n">
-        <v>49.54</v>
+        <v>50.62</v>
       </c>
       <c r="F2" t="n">
-        <v>22.86</v>
+        <v>26.31</v>
       </c>
       <c r="G2" t="n">
-        <v>23.47</v>
+        <v>24.52</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -673,26 +703,26 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.3</v>
+        <v>1.78</v>
       </c>
       <c r="C3" t="n">
-        <v>-1.01</v>
+        <v>0.36</v>
       </c>
       <c r="D3" t="n">
-        <v>10.32</v>
+        <v>7.37</v>
       </c>
       <c r="E3" t="n">
-        <v>11.39</v>
+        <v>9.81</v>
       </c>
       <c r="F3" t="n">
-        <v>9.890000000000001</v>
+        <v>10.21</v>
       </c>
       <c r="G3" t="n">
-        <v>9.31</v>
+        <v>10.12</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -703,26 +733,26 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.95</v>
+        <v>-2.66</v>
       </c>
       <c r="C4" t="n">
-        <v>-1.4</v>
+        <v>-4.58</v>
       </c>
       <c r="D4" t="n">
-        <v>9.24</v>
+        <v>1.61</v>
       </c>
       <c r="E4" t="n">
-        <v>15.03</v>
+        <v>11.08</v>
       </c>
       <c r="F4" t="n">
-        <v>8.84</v>
+        <v>9.16</v>
       </c>
       <c r="G4" t="n">
-        <v>7.91</v>
+        <v>7.51</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -733,26 +763,26 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-3.11</v>
+        <v>-1.78</v>
       </c>
       <c r="C5" t="n">
-        <v>-6.45</v>
+        <v>-7.02</v>
       </c>
       <c r="D5" t="n">
-        <v>10.56</v>
+        <v>6.01</v>
       </c>
       <c r="E5" t="n">
-        <v>10.99</v>
+        <v>8.43</v>
       </c>
       <c r="F5" t="n">
-        <v>10.17</v>
+        <v>9.19</v>
       </c>
       <c r="G5" t="n">
-        <v>2.63</v>
+        <v>2.37</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -763,26 +793,26 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.65</v>
+        <v>-0.6</v>
       </c>
       <c r="C6" t="n">
-        <v>-11.69</v>
+        <v>-5.79</v>
       </c>
       <c r="D6" t="n">
-        <v>4.09</v>
+        <v>-3.42</v>
       </c>
       <c r="E6" t="n">
-        <v>16.41</v>
+        <v>12.59</v>
       </c>
       <c r="F6" t="n">
-        <v>9.32</v>
+        <v>8.19</v>
       </c>
       <c r="G6" t="n">
-        <v>10.45</v>
+        <v>10.61</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -793,26 +823,26 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.77</v>
+        <v>1.63</v>
       </c>
       <c r="C7" t="n">
-        <v>-1.02</v>
+        <v>0.43</v>
       </c>
       <c r="D7" t="n">
-        <v>2.01</v>
+        <v>2.96</v>
       </c>
       <c r="E7" t="n">
-        <v>0.73</v>
+        <v>-0.65</v>
       </c>
       <c r="F7" t="n">
-        <v>1.42</v>
+        <v>1.33</v>
       </c>
       <c r="G7" t="n">
-        <v>6.16</v>
+        <v>6.34</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -823,26 +853,26 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-1.87</v>
+        <v>10.62</v>
       </c>
       <c r="C8" t="n">
-        <v>1.15</v>
+        <v>7.93</v>
       </c>
       <c r="D8" t="n">
-        <v>3.21</v>
+        <v>10.85</v>
       </c>
       <c r="E8" t="n">
-        <v>-2.63</v>
+        <v>0.27</v>
       </c>
       <c r="F8" t="n">
-        <v>6.7</v>
+        <v>8.6</v>
       </c>
       <c r="G8" t="n">
-        <v>4.86</v>
+        <v>6.6</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -853,26 +883,26 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.42</v>
+        <v>-1.43</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.91</v>
+        <v>-4.72</v>
       </c>
       <c r="D9" t="n">
-        <v>12.05</v>
+        <v>4.08</v>
       </c>
       <c r="E9" t="n">
-        <v>18.56</v>
+        <v>15.86</v>
       </c>
       <c r="F9" t="n">
-        <v>16.2</v>
+        <v>15.36</v>
       </c>
       <c r="G9" t="n">
-        <v>8.66</v>
+        <v>9.52</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -883,26 +913,26 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-7.14</v>
+        <v>2.25</v>
       </c>
       <c r="C10" t="n">
-        <v>-9.880000000000001</v>
+        <v>-3.17</v>
       </c>
       <c r="D10" t="n">
-        <v>-23.66</v>
+        <v>-24.37</v>
       </c>
       <c r="E10" t="n">
-        <v>-5.22</v>
+        <v>-5.73</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.87</v>
+        <v>-2.07</v>
       </c>
       <c r="G10" t="n">
-        <v>7.08</v>
+        <v>7.59</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -913,26 +943,26 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.14</v>
+        <v>-0.99</v>
       </c>
       <c r="C11" t="n">
-        <v>-4.56</v>
+        <v>-4.88</v>
       </c>
       <c r="D11" t="n">
-        <v>3.95</v>
+        <v>-1.82</v>
       </c>
       <c r="E11" t="n">
-        <v>12.29</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>9.34</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
-        <v>7.93</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -943,26 +973,26 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-8.68</v>
+        <v>-9.43</v>
       </c>
       <c r="C12" t="n">
-        <v>-26.01</v>
+        <v>-26.86</v>
       </c>
       <c r="D12" t="n">
-        <v>-20.8</v>
+        <v>-31.12</v>
       </c>
       <c r="E12" t="n">
-        <v>15.96</v>
+        <v>10.16</v>
       </c>
       <c r="F12" t="n">
-        <v>0.22</v>
+        <v>-1.82</v>
       </c>
       <c r="G12" t="n">
-        <v>11.64</v>
+        <v>11.19</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -973,26 +1003,26 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.65</v>
+        <v>9.49</v>
       </c>
       <c r="C13" t="n">
-        <v>12.99</v>
+        <v>18.58</v>
       </c>
       <c r="D13" t="n">
-        <v>36.21</v>
+        <v>43.38</v>
       </c>
       <c r="E13" t="n">
-        <v>10.94</v>
+        <v>11.14</v>
       </c>
       <c r="F13" t="n">
-        <v>11.92</v>
+        <v>14.22</v>
       </c>
       <c r="G13" t="n">
-        <v>16.78</v>
+        <v>19.03</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -1003,26 +1033,26 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-1.07</v>
+        <v>0.63</v>
       </c>
       <c r="C14" t="n">
-        <v>-2.58</v>
+        <v>-2.49</v>
       </c>
       <c r="D14" t="n">
-        <v>13.22</v>
+        <v>16.73</v>
       </c>
       <c r="E14" t="n">
-        <v>11.12</v>
+        <v>12.48</v>
       </c>
       <c r="F14" t="n">
-        <v>14.39</v>
+        <v>14.55</v>
       </c>
       <c r="G14" t="n">
-        <v>8.880000000000001</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -1033,26 +1063,26 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10.17</v>
+        <v>3.03</v>
       </c>
       <c r="C15" t="n">
-        <v>8.34</v>
+        <v>12.06</v>
       </c>
       <c r="D15" t="n">
-        <v>39.34</v>
+        <v>43.01</v>
       </c>
       <c r="E15" t="n">
-        <v>17.12</v>
+        <v>15.59</v>
       </c>
       <c r="F15" t="n">
-        <v>12.34</v>
+        <v>12.15</v>
       </c>
       <c r="G15" t="n">
-        <v>13.32</v>
+        <v>14.04</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -1063,26 +1093,26 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-1.23</v>
+        <v>1.01</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>18.35</v>
+        <v>13.24</v>
       </c>
       <c r="E16" t="n">
-        <v>12.75</v>
+        <v>10.96</v>
       </c>
       <c r="F16" t="n">
-        <v>10.27</v>
+        <v>10.73</v>
       </c>
       <c r="G16" t="n">
-        <v>11.95</v>
+        <v>12.47</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -1093,26 +1123,26 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1.42</v>
+        <v>2.74</v>
       </c>
       <c r="C17" t="n">
-        <v>1.8</v>
+        <v>2.65</v>
       </c>
       <c r="D17" t="n">
-        <v>24.96</v>
+        <v>22.76</v>
       </c>
       <c r="E17" t="n">
-        <v>13.44</v>
+        <v>12.08</v>
       </c>
       <c r="F17" t="n">
-        <v>6.85</v>
+        <v>7.49</v>
       </c>
       <c r="G17" t="n">
-        <v>8.640000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -1127,43 +1157,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Fund Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>1 Mth</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>3 Mth</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>1 Yr pa</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>3 Yr pa</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>5 Yr pa</t>
         </is>
       </c>
     </row>
@@ -1185,11 +1220,13 @@
       <c r="E2" t="n">
         <v>35.1903258076034</v>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Auto-fetched by fetch_benchmarks.py</t>
         </is>
+      </c>
+      <c r="H2" t="n">
+        <v>21.27262890808698</v>
       </c>
     </row>
     <row r="3">
@@ -1210,11 +1247,13 @@
       <c r="E3" t="n">
         <v>38.8811110188118</v>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Auto-fetched by fetch_benchmarks.py</t>
         </is>
+      </c>
+      <c r="H3" t="n">
+        <v>25.0481244504585</v>
       </c>
     </row>
     <row r="4">
@@ -1235,11 +1274,13 @@
       <c r="E4" t="n">
         <v>76.1344478370041</v>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Auto-fetched by fetch_benchmarks.py</t>
         </is>
+      </c>
+      <c r="H4" t="n">
+        <v>28.3472807390262</v>
       </c>
     </row>
     <row r="5">
@@ -1260,11 +1301,13 @@
       <c r="E5" t="n">
         <v>33.8241108724727</v>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Auto-fetched by fetch_benchmarks.py</t>
         </is>
+      </c>
+      <c r="H5" t="n">
+        <v>35.93695089645106</v>
       </c>
     </row>
     <row r="6">
@@ -1285,11 +1328,13 @@
       <c r="E6" t="n">
         <v>45.2455665907973</v>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Auto-fetched by fetch_benchmarks.py</t>
         </is>
+      </c>
+      <c r="H6" t="n">
+        <v>23.9844142827319</v>
       </c>
     </row>
     <row r="7">
@@ -1299,24 +1344,27 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2</v>
+        <v>-0.87</v>
       </c>
       <c r="C7" t="n">
-        <v>5.64</v>
+        <v>2.64</v>
       </c>
       <c r="D7" t="n">
-        <v>16.98</v>
+        <v>13.01</v>
       </c>
       <c r="E7" t="n">
-        <v>20.72</v>
-      </c>
-      <c r="F7" s="2" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="F7" s="4" t="n">
         <v>45991</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>Manual if needed</t>
         </is>
+      </c>
+      <c r="H7" t="n">
+        <v>16.11</v>
       </c>
     </row>
     <row r="8">
@@ -1325,12 +1373,6 @@
           <t>Phoenix Growth Fund</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1344,7 +1386,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1353,9 +1395,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1363,9 +1402,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1394,9 +1430,6 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1425,9 +1458,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -1469,9 +1499,6 @@
           <t>• 3 Yr pa = 3-year annualized CPI</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">

</xml_diff>